<commit_message>
Support unmeasured lengths, metre sales and whole coils
</commit_message>
<xml_diff>
--- a/quatt-variants-template.xlsx
+++ b/quatt-variants-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" r:id="R70678239d3854ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как заполнить" sheetId="2" r:id="R5b0485276eaf4ef7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" r:id="Rd712339a8d524b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как заполнить" sheetId="2" r:id="Ref7e136749b9432e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -37,13 +37,33 @@
       <x:sz val="15"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFCE0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3BB"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -73,7 +93,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -102,6 +122,29 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -307,156 +350,226 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="29" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="15" t="str">
         <x:v>Группа вариантов</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="15" t="str">
         <x:v>Артикул карточки</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="15" t="str">
         <x:v>Категория</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="15" t="str">
         <x:v>Диаметр, мм</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
-        <x:v>Длина прутка, м</x:v>
-      </x:c>
-      <x:c r="F1" s="5" t="str">
-        <x:v>Цена за метр</x:v>
-      </x:c>
-      <x:c r="G1" s="5" t="str">
-        <x:v>Закуп за метр</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="E1" s="15" t="str">
+        <x:v>Длина, м</x:v>
+      </x:c>
+      <x:c r="F1" s="15" t="str">
+        <x:v>Цена</x:v>
+      </x:c>
+      <x:c r="G1" s="15" t="str">
+        <x:v>Закуп</x:v>
+      </x:c>
+      <x:c r="H1" s="15" t="str">
         <x:v>Наличие</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="15" t="str">
         <x:v>Единица продажи</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="15" t="str">
         <x:v>Поставщик</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="K1" s="15" t="str">
+        <x:v>Вариант</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="19" t="str">
         <x:v>ПРИМЕР — Арматура А500С</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>EXAMPLE-ARM-A500C</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="str">
-        <x:v>Арматура</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="n">
+      <x:c r="B2" s="19" t="str"/>
+      <x:c r="C2" s="19" t="str">
+        <x:v>Металл</x:v>
+      </x:c>
+      <x:c r="D2" s="20" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="n">
+      <x:c r="E2" s="20" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F2" s="8" t="n">
+      <x:c r="F2" s="20" t="n">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="G2" s="8" t="n">
+      <x:c r="G2" s="20" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="H2" s="7" t="str">
+      <x:c r="H2" s="19" t="str">
         <x:v>Под заказ</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="str">
+      <x:c r="I2" s="19" t="str">
         <x:v>Пруток</x:v>
       </x:c>
-      <x:c r="J2" s="7" t="str"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="7" t="str">
+      <x:c r="J2" s="19" t="str"/>
+      <x:c r="K2" s="19" t="str"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="19" t="str">
         <x:v>ПРИМЕР — Арматура А500С</x:v>
       </x:c>
-      <x:c r="B3" s="7" t="str">
-        <x:v>EXAMPLE-ARM-A500C</x:v>
-      </x:c>
-      <x:c r="C3" s="7" t="str">
-        <x:v>Арматура</x:v>
-      </x:c>
-      <x:c r="D3" s="8" t="n">
+      <x:c r="B3" s="19" t="str"/>
+      <x:c r="C3" s="19" t="str">
+        <x:v>Металл</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E3" s="20" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F3" s="20" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G3" s="20" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="H3" s="19" t="str">
+        <x:v>Под заказ</x:v>
+      </x:c>
+      <x:c r="I3" s="19" t="str">
+        <x:v>Пруток</x:v>
+      </x:c>
+      <x:c r="J3" s="19" t="str"/>
+      <x:c r="K3" s="19" t="str"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="19" t="str">
+        <x:v>ПРИМЕР — Металлический круг</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str"/>
+      <x:c r="C4" s="19" t="str">
+        <x:v>Металл</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="E3" s="8" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="F3" s="8" t="n">
+      <x:c r="E4" s="20" t="str">
+        <x:v>Длина уточняется</x:v>
+      </x:c>
+      <x:c r="F4" s="20" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="G4" s="20" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H4" s="19" t="str">
+        <x:v>Под заказ</x:v>
+      </x:c>
+      <x:c r="I4" s="19" t="str">
+        <x:v>Пруток</x:v>
+      </x:c>
+      <x:c r="J4" s="19" t="str"/>
+      <x:c r="K4" s="19" t="str"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="19" t="str">
+        <x:v>ПРИМЕР — Труба ПНД</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str"/>
+      <x:c r="C5" s="19" t="str">
+        <x:v>Трубы</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E5" s="20" t="str"/>
+      <x:c r="F5" s="20" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G5" s="20" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H5" s="19" t="str">
+        <x:v>Под заказ</x:v>
+      </x:c>
+      <x:c r="I5" s="19" t="str">
+        <x:v>Метр</x:v>
+      </x:c>
+      <x:c r="J5" s="19" t="str"/>
+      <x:c r="K5" s="19" t="str">
+        <x:v>16 мм на отрез</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="19" t="str">
+        <x:v>ПРИМЕР — Труба ПНД</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str"/>
+      <x:c r="C6" s="19" t="str">
+        <x:v>Трубы</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="n">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="G6" s="20" t="n">
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="H6" s="19" t="str">
+        <x:v>Под заказ</x:v>
+      </x:c>
+      <x:c r="I6" s="19" t="str">
+        <x:v>Бухта</x:v>
+      </x:c>
+      <x:c r="J6" s="19" t="str"/>
+      <x:c r="K6" s="19" t="str">
+        <x:v>16 мм, бухта 100 м</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="19" t="str">
+        <x:v>ПРИМЕР — Крепёж</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str"/>
+      <x:c r="C7" s="19" t="str">
+        <x:v>Крепёж</x:v>
+      </x:c>
+      <x:c r="D7" s="20" t="str"/>
+      <x:c r="E7" s="20" t="str"/>
+      <x:c r="F7" s="20" t="n">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="G3" s="8" t="n">
+      <x:c r="G7" s="20" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="H3" s="7" t="str">
+      <x:c r="H7" s="19" t="str">
         <x:v>Под заказ</x:v>
       </x:c>
-      <x:c r="I3" s="7" t="str">
-        <x:v>Пруток</x:v>
-      </x:c>
-      <x:c r="J3" s="7" t="str"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="7" t="str">
-        <x:v>ПРИМЕР — Арматура А500С</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="str">
-        <x:v>EXAMPLE-ARM-A500C</x:v>
-      </x:c>
-      <x:c r="C4" s="7" t="str">
-        <x:v>Арматура</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F4" s="8" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="G4" s="8" t="n">
-        <x:v>380</x:v>
-      </x:c>
-      <x:c r="H4" s="7" t="str">
-        <x:v>Под заказ</x:v>
-      </x:c>
-      <x:c r="I4" s="7" t="str">
-        <x:v>Пруток</x:v>
-      </x:c>
-      <x:c r="J4" s="7" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="D5" s="9"/>
-      <x:c r="E5" s="9"/>
-      <x:c r="F5" s="9"/>
-      <x:c r="G5" s="9"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="D6" s="9"/>
-      <x:c r="E6" s="9"/>
-      <x:c r="F6" s="9"/>
-      <x:c r="G6" s="9"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="D7" s="9"/>
-      <x:c r="E7" s="9"/>
-      <x:c r="F7" s="9"/>
-      <x:c r="G7" s="9"/>
+      <x:c r="I7" s="19" t="str">
+        <x:v>Штука</x:v>
+      </x:c>
+      <x:c r="J7" s="19" t="str"/>
+      <x:c r="K7" s="19" t="str">
+        <x:v>Болт М10</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="D8" s="9"/>
@@ -1028,7 +1141,7 @@
       <x:formula1>"Под заказ,В наличии,Нет в наличии"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:I101">
-      <x:formula1>"Пруток,Штука"</x:formula1>
+      <x:formula1>"Пруток,Штука,Метр,Бухта"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1044,87 +1157,102 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="12" t="str">
-        <x:v>Импорт размеров в каталог QUATT</x:v>
+        <x:v>Импорт товаров и размеров в каталог QUATT</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="13" t="str">
-        <x:v>Пример содержит учебные цены. Замените или удалите все строки с ПРИМЕР.</x:v>
+      <x:c r="A2" s="24" t="str">
+        <x:v>Учебные примеры: замените или удалите все строки с ПРИМЕР. Цены вымышленные.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="11" t="str">
-        <x:v>Заполняйте первый лист «Товары». Первая строка — заголовки, её не удаляйте.</x:v>
+        <x:v>Заполняйте первый лист «Товары». Первую строку с заголовками не удаляйте.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="11" t="str">
-        <x:v>Одна строка — один диаметр и одна длина. 11,7 м и 12 м — две строки.</x:v>
+        <x:v>Единица продажи выбирается в колонке I: Пруток, Штука, Метр или Бухта.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="11" t="str">
-        <x:v>Одинаковая «Группа вариантов» и «Артикул карточки» объединяют строки в одну карточку.</x:v>
+        <x:v>Пруток: цена и закуп за метр; длина — метры одного прутка. Покупатель выбирает целые прутки.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="11" t="str">
-        <x:v>Для новых карточек задайте свой артикул, например ARM-A500C. В дальнейшем его не меняйте.</x:v>
+        <x:v>Метр: цена и закуп за метр. Покупатель может заказать, например, 2,5 м. Длину оставьте пустой.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="str">
-        <x:v>Цена за метр — ваша розничная цена. Закуп за метр — закрытая цена поставщика.</x:v>
+        <x:v>Бухта: цена и закуп за целую бухту. В «Длина, м» укажите метраж одной бухты, например 100.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="str">
-        <x:v>Для прутков укажите диаметр, длину и единицу продажи «Пруток». Количество покупателя — целые прутки.</x:v>
+        <x:v>Штука: цена и закуп за одну штуку. Длина — необязательная характеристика, цену она не умножает.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="str">
-        <x:v>Наличие: Под заказ / В наличии / Нет в наличии. Общие категория и поставщик в одной группе должны совпадать.</x:v>
+        <x:v>Немерная длина: напишите н/м или Длина уточняется. Итог уточняется через WhatsApp; автоматического заказа нет.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="str">
-        <x:v>Не указывайте 6/12 в одной ячейке. Десятичные числа, например 11,7, допустимы.</x:v>
+        <x:v>Одинаковая группа и артикул карточки объединяют строки. Метр и Бухта могут быть вариантами одной карточки.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="str">
-        <x:v>Сайт → Управление → Импорт Excel → выбрать файл → проверить карточки и размеры → Применить выбранное.</x:v>
+        <x:v>Укажите «Вариант» для товаров на метраж и штучных товаров: например «16 мм на отрез» или «Болт М10».</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>Существующие карточки обновляются только после выбора в предпросмотре. Размеры, которых нет в файле, сохраняются.</x:v>
+        <x:v>Артикул необязателен: пустой у нового товара → автоматический QUATT-000001; указанный → ваш артикул.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="11" t="str">
-        <x:v>При обновлении размера пустая цена или закуп сохраняют прежнее значение. Новому размеру нужны обе цены.</x:v>
+        <x:v>Для обновления используйте прежний артикул. Пустая ячейка существующего товара сохраняет его артикул.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="11" t="str">
-        <x:v>Новые карточки по умолчанию скрыты. Добавьте фотографию и проверьте размеры, затем включите показ в каталоге.</x:v>
+        <x:v>Одна строка — один размер и одна длина. 6 м и 12 м — две строки; 11,7 допустимо. Не пишите 6/12 в одной ячейке.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="11" t="str">
-        <x:v>Обычные товары можно импортировать отдельно с колонками Артикул, Название, Категория, Цена, Закуп.</x:v>
+        <x:v>Наличие: Под заказ / В наличии / Нет в наличии. Категория и поставщик внутри группы должны совпадать.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="11" t="str">
-        <x:v>Для вариантов «Штука» добавьте колонку «Вариант». Цена и закуп в этой строке — за штуку. Прутки и штуки храните в разных карточках.</x:v>
+        <x:v>Сайт → Управление → Импорт Excel → выбрать файл → проверить размеры и единицы → Применить выбранное.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="11" t="str">
-        <x:v>Прайсы с объединённой шапкой сначала перенесите в эту таблицу. Цены за тонну не подставляйте в колонку цены за метр.</x:v>
+        <x:v>Существующие товары обновляются только после выбора. Размеры, которых нет в файле, сохраняются.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="11" t="str">
+        <x:v>Пустые цена и закуп сохраняют прежние значения. У нового варианта заполните обе цены.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="11" t="str">
+        <x:v>Новые карточки по умолчанию скрыты. Добавьте фото, проверьте данные и включите показ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="11" t="str">
+        <x:v>Цена за тонну требует пересчёта. Для бухты указывайте цену всей бухты, а не цену за метр или тонну.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>